<commit_message>
feat : tutorial dialouge
</commit_message>
<xml_diff>
--- a/Assets/Excels/CreatureData.xlsx
+++ b/Assets/Excels/CreatureData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devs\TRPG.Client\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E58D80-A899-4697-8996-6012A915813C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78313D57-3971-460B-B56D-BB8D6B467B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreatureData" sheetId="1" r:id="rId1"/>
@@ -49,9 +49,6 @@
     <t># 튜토리얼</t>
   </si>
   <si>
-    <t>SO_Monster_00</t>
-  </si>
-  <si>
     <t>Default</t>
   </si>
   <si>
@@ -64,16 +61,10 @@
     <t>Attack_00</t>
   </si>
   <si>
-    <t>SO_Monster_01</t>
-  </si>
-  <si>
     <t>나이트</t>
   </si>
   <si>
     <t>Knight</t>
-  </si>
-  <si>
-    <t>SO_Monster_02</t>
   </si>
   <si>
     <t>비숍</t>
@@ -82,19 +73,10 @@
     <t>Bishop</t>
   </si>
   <si>
-    <t>SO_Monster_03</t>
-  </si>
-  <si>
     <t>Rook</t>
   </si>
   <si>
-    <t>SO_Monster_04</t>
-  </si>
-  <si>
     <t>Queen</t>
-  </si>
-  <si>
-    <t>SO_Monster_05</t>
   </si>
   <si>
     <t>King</t>
@@ -134,6 +116,30 @@
   </si>
   <si>
     <t>PF_King</t>
+  </si>
+  <si>
+    <t>Monster_00</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster_01</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster_02</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster_03</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster_04</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster_05</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -323,7 +329,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -372,14 +378,585 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="65">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6FAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -397,580 +974,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6FAF7"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -990,7 +993,7 @@
   <autoFilter ref="A1:I200" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
-    <tableColumn id="8" xr3:uid="{FC26B9EF-D3B9-43E3-BEBA-CBD0BF0F99C1}" name="PfId" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{FC26B9EF-D3B9-43E3-BEBA-CBD0BF0F99C1}" name="PfId" dataDxfId="64"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Description"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DisplayName"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Type"/>
@@ -1176,7 +1179,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -1225,22 +1228,22 @@
     </row>
     <row r="3" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="F3" s="14" t="s">
         <v>12</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>13</v>
       </c>
       <c r="G3" s="8">
         <v>10</v>
@@ -1259,22 +1262,22 @@
     </row>
     <row r="4" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>16</v>
-      </c>
       <c r="F4" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G4" s="8">
         <v>10</v>
@@ -1296,22 +1299,22 @@
     </row>
     <row r="5" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
+      <c r="B5" s="7" t="s">
+        <v>26</v>
+      </c>
       <c r="C5" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" s="8">
         <v>10</v>
@@ -1333,22 +1336,22 @@
     </row>
     <row r="6" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>26</v>
-      </c>
       <c r="E6" s="14" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" s="8">
         <v>10</v>
@@ -1370,22 +1373,22 @@
     </row>
     <row r="7" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="16" t="s">
         <v>34</v>
       </c>
+      <c r="B7" s="7" t="s">
+        <v>28</v>
+      </c>
       <c r="C7" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G7" s="8">
         <v>10</v>
@@ -1407,22 +1410,22 @@
     </row>
     <row r="8" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A8" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="16" t="s">
         <v>35</v>
       </c>
+      <c r="B8" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="C8" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G8" s="8">
         <v>10</v>
@@ -1443,7 +1446,7 @@
     </row>
     <row r="9" spans="1:18" ht="14.4" customHeight="1">
       <c r="A9" s="6"/>
-      <c r="B9" s="16"/>
+      <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -1462,7 +1465,7 @@
     </row>
     <row r="10" spans="1:18" ht="14.4" customHeight="1">
       <c r="A10" s="6"/>
-      <c r="B10" s="16"/>
+      <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
@@ -1481,7 +1484,7 @@
     </row>
     <row r="11" spans="1:18" ht="14.4" customHeight="1">
       <c r="A11" s="6"/>
-      <c r="B11" s="16"/>
+      <c r="B11" s="7"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -1500,7 +1503,7 @@
     </row>
     <row r="12" spans="1:18" ht="14.4" customHeight="1">
       <c r="A12" s="6"/>
-      <c r="B12" s="16"/>
+      <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
@@ -1519,7 +1522,7 @@
     </row>
     <row r="13" spans="1:18" ht="14.4" customHeight="1">
       <c r="A13" s="6"/>
-      <c r="B13" s="16"/>
+      <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
@@ -1538,7 +1541,7 @@
     </row>
     <row r="14" spans="1:18" ht="14.4" customHeight="1">
       <c r="A14" s="6"/>
-      <c r="B14" s="16"/>
+      <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
@@ -1557,7 +1560,7 @@
     </row>
     <row r="15" spans="1:18" ht="14.4" customHeight="1">
       <c r="A15" s="6"/>
-      <c r="B15" s="16"/>
+      <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
@@ -1576,7 +1579,7 @@
     </row>
     <row r="16" spans="1:18" ht="14.4" customHeight="1">
       <c r="A16" s="6"/>
-      <c r="B16" s="16"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
@@ -1595,7 +1598,7 @@
     </row>
     <row r="17" spans="1:18" ht="14.4" customHeight="1">
       <c r="A17" s="6"/>
-      <c r="B17" s="16"/>
+      <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
@@ -1614,7 +1617,7 @@
     </row>
     <row r="18" spans="1:18" ht="14.4" customHeight="1">
       <c r="A18" s="6"/>
-      <c r="B18" s="16"/>
+      <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
@@ -1633,7 +1636,7 @@
     </row>
     <row r="19" spans="1:18" ht="14.4" customHeight="1">
       <c r="A19" s="6"/>
-      <c r="B19" s="16"/>
+      <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
@@ -1652,7 +1655,7 @@
     </row>
     <row r="20" spans="1:18" ht="14.4" customHeight="1">
       <c r="A20" s="6"/>
-      <c r="B20" s="16"/>
+      <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
@@ -1671,7 +1674,7 @@
     </row>
     <row r="21" spans="1:18" ht="14.4" customHeight="1">
       <c r="A21" s="6"/>
-      <c r="B21" s="16"/>
+      <c r="B21" s="7"/>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
@@ -1690,7 +1693,7 @@
     </row>
     <row r="22" spans="1:18" ht="14.4" customHeight="1">
       <c r="A22" s="6"/>
-      <c r="B22" s="16"/>
+      <c r="B22" s="7"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
       <c r="E22" s="7"/>
@@ -1709,7 +1712,7 @@
     </row>
     <row r="23" spans="1:18" ht="14.4" customHeight="1">
       <c r="A23" s="6"/>
-      <c r="B23" s="16"/>
+      <c r="B23" s="7"/>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
@@ -1728,7 +1731,7 @@
     </row>
     <row r="24" spans="1:18" ht="14.4" customHeight="1">
       <c r="A24" s="6"/>
-      <c r="B24" s="16"/>
+      <c r="B24" s="7"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="7"/>
@@ -1747,7 +1750,7 @@
     </row>
     <row r="25" spans="1:18" ht="14.4" customHeight="1">
       <c r="A25" s="6"/>
-      <c r="B25" s="16"/>
+      <c r="B25" s="7"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
@@ -1766,7 +1769,7 @@
     </row>
     <row r="26" spans="1:18" ht="14.4" customHeight="1">
       <c r="A26" s="6"/>
-      <c r="B26" s="16"/>
+      <c r="B26" s="7"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
@@ -1785,7 +1788,7 @@
     </row>
     <row r="27" spans="1:18" ht="14.4" customHeight="1">
       <c r="A27" s="6"/>
-      <c r="B27" s="16"/>
+      <c r="B27" s="7"/>
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
       <c r="E27" s="7"/>
@@ -1804,7 +1807,7 @@
     </row>
     <row r="28" spans="1:18" ht="14.4" customHeight="1">
       <c r="A28" s="6"/>
-      <c r="B28" s="16"/>
+      <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
@@ -1823,7 +1826,7 @@
     </row>
     <row r="29" spans="1:18" ht="14.4" customHeight="1">
       <c r="A29" s="6"/>
-      <c r="B29" s="16"/>
+      <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
@@ -1842,7 +1845,7 @@
     </row>
     <row r="30" spans="1:18" ht="14.4" customHeight="1">
       <c r="A30" s="6"/>
-      <c r="B30" s="16"/>
+      <c r="B30" s="7"/>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
@@ -1861,7 +1864,7 @@
     </row>
     <row r="31" spans="1:18" ht="14.4" customHeight="1">
       <c r="A31" s="6"/>
-      <c r="B31" s="16"/>
+      <c r="B31" s="7"/>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
@@ -1880,7 +1883,7 @@
     </row>
     <row r="32" spans="1:18" ht="14.4" customHeight="1">
       <c r="A32" s="6"/>
-      <c r="B32" s="16"/>
+      <c r="B32" s="7"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
@@ -1899,7 +1902,7 @@
     </row>
     <row r="33" spans="1:18" ht="14.4" customHeight="1">
       <c r="A33" s="6"/>
-      <c r="B33" s="16"/>
+      <c r="B33" s="7"/>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
@@ -1918,7 +1921,7 @@
     </row>
     <row r="34" spans="1:18" ht="14.4" customHeight="1">
       <c r="A34" s="6"/>
-      <c r="B34" s="16"/>
+      <c r="B34" s="7"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
@@ -1937,7 +1940,7 @@
     </row>
     <row r="35" spans="1:18" ht="14.4" customHeight="1">
       <c r="A35" s="6"/>
-      <c r="B35" s="16"/>
+      <c r="B35" s="7"/>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
@@ -1956,7 +1959,7 @@
     </row>
     <row r="36" spans="1:18" ht="14.4" customHeight="1">
       <c r="A36" s="6"/>
-      <c r="B36" s="16"/>
+      <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
@@ -1975,7 +1978,7 @@
     </row>
     <row r="37" spans="1:18" ht="14.4" customHeight="1">
       <c r="A37" s="6"/>
-      <c r="B37" s="16"/>
+      <c r="B37" s="7"/>
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
@@ -1994,7 +1997,7 @@
     </row>
     <row r="38" spans="1:18" ht="14.4" customHeight="1">
       <c r="A38" s="6"/>
-      <c r="B38" s="16"/>
+      <c r="B38" s="7"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
@@ -2013,7 +2016,7 @@
     </row>
     <row r="39" spans="1:18" ht="14.4" customHeight="1">
       <c r="A39" s="6"/>
-      <c r="B39" s="16"/>
+      <c r="B39" s="7"/>
       <c r="C39" s="7"/>
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
@@ -2032,7 +2035,7 @@
     </row>
     <row r="40" spans="1:18" ht="14.4" customHeight="1">
       <c r="A40" s="6"/>
-      <c r="B40" s="16"/>
+      <c r="B40" s="7"/>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
       <c r="E40" s="7"/>
@@ -2051,7 +2054,7 @@
     </row>
     <row r="41" spans="1:18" ht="14.4" customHeight="1">
       <c r="A41" s="6"/>
-      <c r="B41" s="16"/>
+      <c r="B41" s="7"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
@@ -2070,7 +2073,7 @@
     </row>
     <row r="42" spans="1:18" ht="14.4" customHeight="1">
       <c r="A42" s="6"/>
-      <c r="B42" s="16"/>
+      <c r="B42" s="7"/>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
       <c r="E42" s="7"/>
@@ -2089,7 +2092,7 @@
     </row>
     <row r="43" spans="1:18" ht="14.4" customHeight="1">
       <c r="A43" s="6"/>
-      <c r="B43" s="16"/>
+      <c r="B43" s="7"/>
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
       <c r="E43" s="7"/>
@@ -2108,7 +2111,7 @@
     </row>
     <row r="44" spans="1:18" ht="14.4" customHeight="1">
       <c r="A44" s="6"/>
-      <c r="B44" s="16"/>
+      <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
       <c r="E44" s="7"/>
@@ -2127,7 +2130,7 @@
     </row>
     <row r="45" spans="1:18" ht="14.4" customHeight="1">
       <c r="A45" s="6"/>
-      <c r="B45" s="16"/>
+      <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7"/>
@@ -2146,7 +2149,7 @@
     </row>
     <row r="46" spans="1:18" ht="14.4" customHeight="1">
       <c r="A46" s="6"/>
-      <c r="B46" s="16"/>
+      <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
@@ -2165,7 +2168,7 @@
     </row>
     <row r="47" spans="1:18" ht="14.4" customHeight="1">
       <c r="A47" s="6"/>
-      <c r="B47" s="16"/>
+      <c r="B47" s="7"/>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
@@ -2184,7 +2187,7 @@
     </row>
     <row r="48" spans="1:18" ht="14.4" customHeight="1">
       <c r="A48" s="6"/>
-      <c r="B48" s="16"/>
+      <c r="B48" s="7"/>
       <c r="C48" s="7"/>
       <c r="D48" s="7"/>
       <c r="E48" s="7"/>
@@ -2203,7 +2206,7 @@
     </row>
     <row r="49" spans="1:18" ht="14.4" customHeight="1">
       <c r="A49" s="6"/>
-      <c r="B49" s="16"/>
+      <c r="B49" s="7"/>
       <c r="C49" s="7"/>
       <c r="D49" s="7"/>
       <c r="E49" s="7"/>
@@ -2222,7 +2225,7 @@
     </row>
     <row r="50" spans="1:18" ht="14.4" customHeight="1">
       <c r="A50" s="6"/>
-      <c r="B50" s="16"/>
+      <c r="B50" s="7"/>
       <c r="C50" s="7"/>
       <c r="D50" s="7"/>
       <c r="E50" s="7"/>
@@ -2241,7 +2244,7 @@
     </row>
     <row r="51" spans="1:18" ht="14.4" customHeight="1">
       <c r="A51" s="6"/>
-      <c r="B51" s="16"/>
+      <c r="B51" s="7"/>
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
@@ -2260,7 +2263,7 @@
     </row>
     <row r="52" spans="1:18" ht="14.4" customHeight="1">
       <c r="A52" s="6"/>
-      <c r="B52" s="16"/>
+      <c r="B52" s="7"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
@@ -2279,7 +2282,7 @@
     </row>
     <row r="53" spans="1:18" ht="14.4" customHeight="1">
       <c r="A53" s="6"/>
-      <c r="B53" s="16"/>
+      <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
@@ -2298,7 +2301,7 @@
     </row>
     <row r="54" spans="1:18" ht="14.4" customHeight="1">
       <c r="A54" s="6"/>
-      <c r="B54" s="16"/>
+      <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
@@ -2317,7 +2320,7 @@
     </row>
     <row r="55" spans="1:18" ht="14.4" customHeight="1">
       <c r="A55" s="6"/>
-      <c r="B55" s="16"/>
+      <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
       <c r="E55" s="7"/>
@@ -2336,7 +2339,7 @@
     </row>
     <row r="56" spans="1:18" ht="14.4" customHeight="1">
       <c r="A56" s="6"/>
-      <c r="B56" s="16"/>
+      <c r="B56" s="7"/>
       <c r="C56" s="7"/>
       <c r="D56" s="7"/>
       <c r="E56" s="7"/>
@@ -2355,7 +2358,7 @@
     </row>
     <row r="57" spans="1:18" ht="14.4" customHeight="1">
       <c r="A57" s="6"/>
-      <c r="B57" s="16"/>
+      <c r="B57" s="7"/>
       <c r="C57" s="7"/>
       <c r="D57" s="7"/>
       <c r="E57" s="7"/>
@@ -2374,7 +2377,7 @@
     </row>
     <row r="58" spans="1:18" ht="14.4" customHeight="1">
       <c r="A58" s="6"/>
-      <c r="B58" s="16"/>
+      <c r="B58" s="7"/>
       <c r="C58" s="7"/>
       <c r="D58" s="7"/>
       <c r="E58" s="7"/>
@@ -2393,7 +2396,7 @@
     </row>
     <row r="59" spans="1:18" ht="14.4" customHeight="1">
       <c r="A59" s="6"/>
-      <c r="B59" s="16"/>
+      <c r="B59" s="7"/>
       <c r="C59" s="7"/>
       <c r="D59" s="7"/>
       <c r="E59" s="7"/>
@@ -2412,7 +2415,7 @@
     </row>
     <row r="60" spans="1:18" ht="14.4" customHeight="1">
       <c r="A60" s="6"/>
-      <c r="B60" s="16"/>
+      <c r="B60" s="7"/>
       <c r="C60" s="7"/>
       <c r="D60" s="7"/>
       <c r="E60" s="7"/>
@@ -2431,7 +2434,7 @@
     </row>
     <row r="61" spans="1:18" ht="14.4" customHeight="1">
       <c r="A61" s="6"/>
-      <c r="B61" s="16"/>
+      <c r="B61" s="7"/>
       <c r="C61" s="7"/>
       <c r="D61" s="7"/>
       <c r="E61" s="7"/>
@@ -2450,7 +2453,7 @@
     </row>
     <row r="62" spans="1:18" ht="14.4" customHeight="1">
       <c r="A62" s="6"/>
-      <c r="B62" s="16"/>
+      <c r="B62" s="7"/>
       <c r="C62" s="7"/>
       <c r="D62" s="7"/>
       <c r="E62" s="7"/>
@@ -2469,7 +2472,7 @@
     </row>
     <row r="63" spans="1:18" ht="14.4" customHeight="1">
       <c r="A63" s="6"/>
-      <c r="B63" s="16"/>
+      <c r="B63" s="7"/>
       <c r="C63" s="7"/>
       <c r="D63" s="7"/>
       <c r="E63" s="7"/>
@@ -2488,7 +2491,7 @@
     </row>
     <row r="64" spans="1:18" ht="14.4" customHeight="1">
       <c r="A64" s="6"/>
-      <c r="B64" s="16"/>
+      <c r="B64" s="7"/>
       <c r="C64" s="7"/>
       <c r="D64" s="7"/>
       <c r="E64" s="7"/>
@@ -2507,7 +2510,7 @@
     </row>
     <row r="65" spans="1:18" ht="14.4" customHeight="1">
       <c r="A65" s="6"/>
-      <c r="B65" s="16"/>
+      <c r="B65" s="7"/>
       <c r="C65" s="7"/>
       <c r="D65" s="7"/>
       <c r="E65" s="7"/>
@@ -2526,7 +2529,7 @@
     </row>
     <row r="66" spans="1:18" ht="14.4" customHeight="1">
       <c r="A66" s="6"/>
-      <c r="B66" s="16"/>
+      <c r="B66" s="7"/>
       <c r="C66" s="7"/>
       <c r="D66" s="7"/>
       <c r="E66" s="7"/>
@@ -2545,7 +2548,7 @@
     </row>
     <row r="67" spans="1:18" ht="14.4" customHeight="1">
       <c r="A67" s="6"/>
-      <c r="B67" s="16"/>
+      <c r="B67" s="7"/>
       <c r="C67" s="7"/>
       <c r="D67" s="7"/>
       <c r="E67" s="7"/>
@@ -2564,7 +2567,7 @@
     </row>
     <row r="68" spans="1:18" ht="14.4" customHeight="1">
       <c r="A68" s="6"/>
-      <c r="B68" s="16"/>
+      <c r="B68" s="7"/>
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
       <c r="E68" s="7"/>
@@ -2583,7 +2586,7 @@
     </row>
     <row r="69" spans="1:18" ht="14.4" customHeight="1">
       <c r="A69" s="6"/>
-      <c r="B69" s="16"/>
+      <c r="B69" s="7"/>
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
       <c r="E69" s="7"/>
@@ -2602,7 +2605,7 @@
     </row>
     <row r="70" spans="1:18" ht="14.4" customHeight="1">
       <c r="A70" s="6"/>
-      <c r="B70" s="16"/>
+      <c r="B70" s="7"/>
       <c r="C70" s="7"/>
       <c r="D70" s="7"/>
       <c r="E70" s="7"/>
@@ -2621,7 +2624,7 @@
     </row>
     <row r="71" spans="1:18" ht="14.4" customHeight="1">
       <c r="A71" s="6"/>
-      <c r="B71" s="16"/>
+      <c r="B71" s="7"/>
       <c r="C71" s="7"/>
       <c r="D71" s="7"/>
       <c r="E71" s="7"/>
@@ -2640,7 +2643,7 @@
     </row>
     <row r="72" spans="1:18" ht="14.4" customHeight="1">
       <c r="A72" s="6"/>
-      <c r="B72" s="16"/>
+      <c r="B72" s="7"/>
       <c r="C72" s="7"/>
       <c r="D72" s="7"/>
       <c r="E72" s="7"/>
@@ -2659,7 +2662,7 @@
     </row>
     <row r="73" spans="1:18" ht="14.4" customHeight="1">
       <c r="A73" s="6"/>
-      <c r="B73" s="16"/>
+      <c r="B73" s="7"/>
       <c r="C73" s="7"/>
       <c r="D73" s="7"/>
       <c r="E73" s="7"/>
@@ -2678,7 +2681,7 @@
     </row>
     <row r="74" spans="1:18" ht="14.4" customHeight="1">
       <c r="A74" s="6"/>
-      <c r="B74" s="16"/>
+      <c r="B74" s="7"/>
       <c r="C74" s="7"/>
       <c r="D74" s="7"/>
       <c r="E74" s="7"/>
@@ -2697,7 +2700,7 @@
     </row>
     <row r="75" spans="1:18" ht="14.4" customHeight="1">
       <c r="A75" s="6"/>
-      <c r="B75" s="16"/>
+      <c r="B75" s="7"/>
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
@@ -2716,7 +2719,7 @@
     </row>
     <row r="76" spans="1:18" ht="14.4" customHeight="1">
       <c r="A76" s="6"/>
-      <c r="B76" s="16"/>
+      <c r="B76" s="7"/>
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
       <c r="E76" s="7"/>
@@ -2735,7 +2738,7 @@
     </row>
     <row r="77" spans="1:18" ht="14.4" customHeight="1">
       <c r="A77" s="6"/>
-      <c r="B77" s="16"/>
+      <c r="B77" s="7"/>
       <c r="C77" s="7"/>
       <c r="D77" s="7"/>
       <c r="E77" s="7"/>
@@ -2754,7 +2757,7 @@
     </row>
     <row r="78" spans="1:18" ht="14.4" customHeight="1">
       <c r="A78" s="6"/>
-      <c r="B78" s="16"/>
+      <c r="B78" s="7"/>
       <c r="C78" s="7"/>
       <c r="D78" s="7"/>
       <c r="E78" s="7"/>
@@ -2773,7 +2776,7 @@
     </row>
     <row r="79" spans="1:18" ht="14.4" customHeight="1">
       <c r="A79" s="6"/>
-      <c r="B79" s="16"/>
+      <c r="B79" s="7"/>
       <c r="C79" s="7"/>
       <c r="D79" s="7"/>
       <c r="E79" s="7"/>
@@ -2792,7 +2795,7 @@
     </row>
     <row r="80" spans="1:18" ht="14.4" customHeight="1">
       <c r="A80" s="6"/>
-      <c r="B80" s="16"/>
+      <c r="B80" s="7"/>
       <c r="C80" s="7"/>
       <c r="D80" s="7"/>
       <c r="E80" s="7"/>
@@ -2811,7 +2814,7 @@
     </row>
     <row r="81" spans="1:18" ht="14.4" customHeight="1">
       <c r="A81" s="6"/>
-      <c r="B81" s="16"/>
+      <c r="B81" s="7"/>
       <c r="C81" s="7"/>
       <c r="D81" s="7"/>
       <c r="E81" s="7"/>
@@ -2830,7 +2833,7 @@
     </row>
     <row r="82" spans="1:18" ht="14.4" customHeight="1">
       <c r="A82" s="6"/>
-      <c r="B82" s="16"/>
+      <c r="B82" s="7"/>
       <c r="C82" s="7"/>
       <c r="D82" s="7"/>
       <c r="E82" s="7"/>
@@ -2849,7 +2852,7 @@
     </row>
     <row r="83" spans="1:18" ht="14.4" customHeight="1">
       <c r="A83" s="6"/>
-      <c r="B83" s="16"/>
+      <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
@@ -2868,7 +2871,7 @@
     </row>
     <row r="84" spans="1:18" ht="14.4" customHeight="1">
       <c r="A84" s="6"/>
-      <c r="B84" s="16"/>
+      <c r="B84" s="7"/>
       <c r="C84" s="7"/>
       <c r="D84" s="7"/>
       <c r="E84" s="7"/>
@@ -2887,7 +2890,7 @@
     </row>
     <row r="85" spans="1:18" ht="14.4" customHeight="1">
       <c r="A85" s="6"/>
-      <c r="B85" s="16"/>
+      <c r="B85" s="7"/>
       <c r="C85" s="7"/>
       <c r="D85" s="7"/>
       <c r="E85" s="7"/>
@@ -2906,7 +2909,7 @@
     </row>
     <row r="86" spans="1:18" ht="14.4" customHeight="1">
       <c r="A86" s="6"/>
-      <c r="B86" s="16"/>
+      <c r="B86" s="7"/>
       <c r="C86" s="7"/>
       <c r="D86" s="7"/>
       <c r="E86" s="7"/>
@@ -2925,7 +2928,7 @@
     </row>
     <row r="87" spans="1:18" ht="14.4" customHeight="1">
       <c r="A87" s="6"/>
-      <c r="B87" s="16"/>
+      <c r="B87" s="7"/>
       <c r="C87" s="7"/>
       <c r="D87" s="7"/>
       <c r="E87" s="7"/>
@@ -2944,7 +2947,7 @@
     </row>
     <row r="88" spans="1:18" ht="14.4" customHeight="1">
       <c r="A88" s="6"/>
-      <c r="B88" s="16"/>
+      <c r="B88" s="7"/>
       <c r="C88" s="7"/>
       <c r="D88" s="7"/>
       <c r="E88" s="7"/>
@@ -2963,7 +2966,7 @@
     </row>
     <row r="89" spans="1:18" ht="14.4" customHeight="1">
       <c r="A89" s="6"/>
-      <c r="B89" s="16"/>
+      <c r="B89" s="7"/>
       <c r="C89" s="7"/>
       <c r="D89" s="7"/>
       <c r="E89" s="7"/>
@@ -2982,7 +2985,7 @@
     </row>
     <row r="90" spans="1:18" ht="14.4" customHeight="1">
       <c r="A90" s="6"/>
-      <c r="B90" s="16"/>
+      <c r="B90" s="7"/>
       <c r="C90" s="7"/>
       <c r="D90" s="7"/>
       <c r="E90" s="7"/>
@@ -3001,7 +3004,7 @@
     </row>
     <row r="91" spans="1:18" ht="14.4" customHeight="1">
       <c r="A91" s="6"/>
-      <c r="B91" s="16"/>
+      <c r="B91" s="7"/>
       <c r="C91" s="7"/>
       <c r="D91" s="7"/>
       <c r="E91" s="7"/>
@@ -3020,7 +3023,7 @@
     </row>
     <row r="92" spans="1:18" ht="14.4" customHeight="1">
       <c r="A92" s="6"/>
-      <c r="B92" s="16"/>
+      <c r="B92" s="7"/>
       <c r="C92" s="7"/>
       <c r="D92" s="7"/>
       <c r="E92" s="7"/>
@@ -3039,7 +3042,7 @@
     </row>
     <row r="93" spans="1:18" ht="14.4" customHeight="1">
       <c r="A93" s="6"/>
-      <c r="B93" s="16"/>
+      <c r="B93" s="7"/>
       <c r="C93" s="7"/>
       <c r="D93" s="7"/>
       <c r="E93" s="7"/>
@@ -3058,7 +3061,7 @@
     </row>
     <row r="94" spans="1:18" ht="14.4" customHeight="1">
       <c r="A94" s="6"/>
-      <c r="B94" s="16"/>
+      <c r="B94" s="7"/>
       <c r="C94" s="7"/>
       <c r="D94" s="7"/>
       <c r="E94" s="7"/>
@@ -3077,7 +3080,7 @@
     </row>
     <row r="95" spans="1:18" ht="14.4" customHeight="1">
       <c r="A95" s="6"/>
-      <c r="B95" s="16"/>
+      <c r="B95" s="7"/>
       <c r="C95" s="7"/>
       <c r="D95" s="7"/>
       <c r="E95" s="7"/>
@@ -3096,7 +3099,7 @@
     </row>
     <row r="96" spans="1:18" ht="14.4" customHeight="1">
       <c r="A96" s="6"/>
-      <c r="B96" s="16"/>
+      <c r="B96" s="7"/>
       <c r="C96" s="7"/>
       <c r="D96" s="7"/>
       <c r="E96" s="7"/>
@@ -3115,7 +3118,7 @@
     </row>
     <row r="97" spans="1:18" ht="14.4" customHeight="1">
       <c r="A97" s="6"/>
-      <c r="B97" s="16"/>
+      <c r="B97" s="7"/>
       <c r="C97" s="7"/>
       <c r="D97" s="7"/>
       <c r="E97" s="7"/>
@@ -3134,7 +3137,7 @@
     </row>
     <row r="98" spans="1:18" ht="14.4" customHeight="1">
       <c r="A98" s="6"/>
-      <c r="B98" s="16"/>
+      <c r="B98" s="7"/>
       <c r="C98" s="7"/>
       <c r="D98" s="7"/>
       <c r="E98" s="7"/>
@@ -3153,7 +3156,7 @@
     </row>
     <row r="99" spans="1:18" ht="14.4" customHeight="1">
       <c r="A99" s="6"/>
-      <c r="B99" s="16"/>
+      <c r="B99" s="7"/>
       <c r="C99" s="7"/>
       <c r="D99" s="7"/>
       <c r="E99" s="7"/>
@@ -3172,7 +3175,7 @@
     </row>
     <row r="100" spans="1:18" ht="14.4" customHeight="1">
       <c r="A100" s="6"/>
-      <c r="B100" s="16"/>
+      <c r="B100" s="7"/>
       <c r="C100" s="7"/>
       <c r="D100" s="7"/>
       <c r="E100" s="7"/>
@@ -3191,7 +3194,7 @@
     </row>
     <row r="101" spans="1:18" ht="14.4" customHeight="1">
       <c r="A101" s="6"/>
-      <c r="B101" s="16"/>
+      <c r="B101" s="7"/>
       <c r="C101" s="7"/>
       <c r="D101" s="7"/>
       <c r="E101" s="7"/>
@@ -3210,7 +3213,7 @@
     </row>
     <row r="102" spans="1:18" ht="14.4" customHeight="1">
       <c r="A102" s="6"/>
-      <c r="B102" s="16"/>
+      <c r="B102" s="7"/>
       <c r="C102" s="7"/>
       <c r="D102" s="7"/>
       <c r="E102" s="7"/>
@@ -3229,7 +3232,7 @@
     </row>
     <row r="103" spans="1:18" ht="14.4" customHeight="1">
       <c r="A103" s="6"/>
-      <c r="B103" s="16"/>
+      <c r="B103" s="7"/>
       <c r="C103" s="7"/>
       <c r="D103" s="7"/>
       <c r="E103" s="7"/>
@@ -3248,7 +3251,7 @@
     </row>
     <row r="104" spans="1:18" ht="14.4" customHeight="1">
       <c r="A104" s="6"/>
-      <c r="B104" s="16"/>
+      <c r="B104" s="7"/>
       <c r="C104" s="7"/>
       <c r="D104" s="7"/>
       <c r="E104" s="7"/>
@@ -3267,7 +3270,7 @@
     </row>
     <row r="105" spans="1:18" ht="14.4" customHeight="1">
       <c r="A105" s="6"/>
-      <c r="B105" s="16"/>
+      <c r="B105" s="7"/>
       <c r="C105" s="7"/>
       <c r="D105" s="7"/>
       <c r="E105" s="7"/>
@@ -3286,7 +3289,7 @@
     </row>
     <row r="106" spans="1:18" ht="14.4" customHeight="1">
       <c r="A106" s="6"/>
-      <c r="B106" s="16"/>
+      <c r="B106" s="7"/>
       <c r="C106" s="7"/>
       <c r="D106" s="7"/>
       <c r="E106" s="7"/>
@@ -3305,7 +3308,7 @@
     </row>
     <row r="107" spans="1:18" ht="14.4" customHeight="1">
       <c r="A107" s="6"/>
-      <c r="B107" s="16"/>
+      <c r="B107" s="7"/>
       <c r="C107" s="7"/>
       <c r="D107" s="7"/>
       <c r="E107" s="7"/>
@@ -3324,7 +3327,7 @@
     </row>
     <row r="108" spans="1:18" ht="14.4" customHeight="1">
       <c r="A108" s="6"/>
-      <c r="B108" s="16"/>
+      <c r="B108" s="7"/>
       <c r="C108" s="7"/>
       <c r="D108" s="7"/>
       <c r="E108" s="7"/>
@@ -3343,7 +3346,7 @@
     </row>
     <row r="109" spans="1:18" ht="14.4" customHeight="1">
       <c r="A109" s="6"/>
-      <c r="B109" s="16"/>
+      <c r="B109" s="7"/>
       <c r="C109" s="7"/>
       <c r="D109" s="7"/>
       <c r="E109" s="7"/>
@@ -3362,7 +3365,7 @@
     </row>
     <row r="110" spans="1:18" ht="14.4" customHeight="1">
       <c r="A110" s="6"/>
-      <c r="B110" s="16"/>
+      <c r="B110" s="7"/>
       <c r="C110" s="7"/>
       <c r="D110" s="7"/>
       <c r="E110" s="7"/>
@@ -3381,7 +3384,7 @@
     </row>
     <row r="111" spans="1:18" ht="14.4" customHeight="1">
       <c r="A111" s="6"/>
-      <c r="B111" s="16"/>
+      <c r="B111" s="7"/>
       <c r="C111" s="7"/>
       <c r="D111" s="7"/>
       <c r="E111" s="7"/>
@@ -3400,7 +3403,7 @@
     </row>
     <row r="112" spans="1:18" ht="14.4" customHeight="1">
       <c r="A112" s="6"/>
-      <c r="B112" s="16"/>
+      <c r="B112" s="7"/>
       <c r="C112" s="7"/>
       <c r="D112" s="7"/>
       <c r="E112" s="7"/>
@@ -3419,7 +3422,7 @@
     </row>
     <row r="113" spans="1:18" ht="14.4" customHeight="1">
       <c r="A113" s="6"/>
-      <c r="B113" s="16"/>
+      <c r="B113" s="7"/>
       <c r="C113" s="7"/>
       <c r="D113" s="7"/>
       <c r="E113" s="7"/>
@@ -3438,7 +3441,7 @@
     </row>
     <row r="114" spans="1:18" ht="14.4" customHeight="1">
       <c r="A114" s="6"/>
-      <c r="B114" s="16"/>
+      <c r="B114" s="7"/>
       <c r="C114" s="7"/>
       <c r="D114" s="7"/>
       <c r="E114" s="7"/>
@@ -3457,7 +3460,7 @@
     </row>
     <row r="115" spans="1:18" ht="14.4" customHeight="1">
       <c r="A115" s="6"/>
-      <c r="B115" s="16"/>
+      <c r="B115" s="7"/>
       <c r="C115" s="7"/>
       <c r="D115" s="7"/>
       <c r="E115" s="7"/>
@@ -3476,7 +3479,7 @@
     </row>
     <row r="116" spans="1:18" ht="14.4" customHeight="1">
       <c r="A116" s="6"/>
-      <c r="B116" s="16"/>
+      <c r="B116" s="7"/>
       <c r="C116" s="7"/>
       <c r="D116" s="7"/>
       <c r="E116" s="7"/>
@@ -3495,7 +3498,7 @@
     </row>
     <row r="117" spans="1:18" ht="14.4" customHeight="1">
       <c r="A117" s="6"/>
-      <c r="B117" s="16"/>
+      <c r="B117" s="7"/>
       <c r="C117" s="7"/>
       <c r="D117" s="7"/>
       <c r="E117" s="7"/>
@@ -3514,7 +3517,7 @@
     </row>
     <row r="118" spans="1:18" ht="14.4" customHeight="1">
       <c r="A118" s="6"/>
-      <c r="B118" s="16"/>
+      <c r="B118" s="7"/>
       <c r="C118" s="7"/>
       <c r="D118" s="7"/>
       <c r="E118" s="7"/>
@@ -3533,7 +3536,7 @@
     </row>
     <row r="119" spans="1:18" ht="14.4" customHeight="1">
       <c r="A119" s="6"/>
-      <c r="B119" s="16"/>
+      <c r="B119" s="7"/>
       <c r="C119" s="7"/>
       <c r="D119" s="7"/>
       <c r="E119" s="7"/>
@@ -3552,7 +3555,7 @@
     </row>
     <row r="120" spans="1:18" ht="14.4" customHeight="1">
       <c r="A120" s="6"/>
-      <c r="B120" s="16"/>
+      <c r="B120" s="7"/>
       <c r="C120" s="7"/>
       <c r="D120" s="7"/>
       <c r="E120" s="7"/>
@@ -3571,7 +3574,7 @@
     </row>
     <row r="121" spans="1:18" ht="14.4" customHeight="1">
       <c r="A121" s="6"/>
-      <c r="B121" s="16"/>
+      <c r="B121" s="7"/>
       <c r="C121" s="7"/>
       <c r="D121" s="7"/>
       <c r="E121" s="7"/>
@@ -3590,7 +3593,7 @@
     </row>
     <row r="122" spans="1:18" ht="14.4" customHeight="1">
       <c r="A122" s="6"/>
-      <c r="B122" s="16"/>
+      <c r="B122" s="7"/>
       <c r="C122" s="7"/>
       <c r="D122" s="7"/>
       <c r="E122" s="7"/>
@@ -3609,7 +3612,7 @@
     </row>
     <row r="123" spans="1:18" ht="14.4" customHeight="1">
       <c r="A123" s="6"/>
-      <c r="B123" s="16"/>
+      <c r="B123" s="7"/>
       <c r="C123" s="7"/>
       <c r="D123" s="7"/>
       <c r="E123" s="7"/>
@@ -3628,7 +3631,7 @@
     </row>
     <row r="124" spans="1:18" ht="14.4" customHeight="1">
       <c r="A124" s="6"/>
-      <c r="B124" s="16"/>
+      <c r="B124" s="7"/>
       <c r="C124" s="7"/>
       <c r="D124" s="7"/>
       <c r="E124" s="7"/>
@@ -3647,7 +3650,7 @@
     </row>
     <row r="125" spans="1:18" ht="14.4" customHeight="1">
       <c r="A125" s="6"/>
-      <c r="B125" s="16"/>
+      <c r="B125" s="7"/>
       <c r="C125" s="7"/>
       <c r="D125" s="7"/>
       <c r="E125" s="7"/>
@@ -3666,7 +3669,7 @@
     </row>
     <row r="126" spans="1:18" ht="14.4" customHeight="1">
       <c r="A126" s="6"/>
-      <c r="B126" s="16"/>
+      <c r="B126" s="7"/>
       <c r="C126" s="7"/>
       <c r="D126" s="7"/>
       <c r="E126" s="7"/>
@@ -3685,7 +3688,7 @@
     </row>
     <row r="127" spans="1:18" ht="14.4" customHeight="1">
       <c r="A127" s="6"/>
-      <c r="B127" s="16"/>
+      <c r="B127" s="7"/>
       <c r="C127" s="7"/>
       <c r="D127" s="7"/>
       <c r="E127" s="7"/>
@@ -3704,7 +3707,7 @@
     </row>
     <row r="128" spans="1:18" ht="14.4" customHeight="1">
       <c r="A128" s="6"/>
-      <c r="B128" s="16"/>
+      <c r="B128" s="7"/>
       <c r="C128" s="7"/>
       <c r="D128" s="7"/>
       <c r="E128" s="7"/>
@@ -3723,7 +3726,7 @@
     </row>
     <row r="129" spans="1:18" ht="14.4" customHeight="1">
       <c r="A129" s="6"/>
-      <c r="B129" s="16"/>
+      <c r="B129" s="7"/>
       <c r="C129" s="7"/>
       <c r="D129" s="7"/>
       <c r="E129" s="7"/>
@@ -3742,7 +3745,7 @@
     </row>
     <row r="130" spans="1:18" ht="14.4" customHeight="1">
       <c r="A130" s="6"/>
-      <c r="B130" s="16"/>
+      <c r="B130" s="7"/>
       <c r="C130" s="7"/>
       <c r="D130" s="7"/>
       <c r="E130" s="7"/>
@@ -3761,7 +3764,7 @@
     </row>
     <row r="131" spans="1:18" ht="14.4" customHeight="1">
       <c r="A131" s="6"/>
-      <c r="B131" s="16"/>
+      <c r="B131" s="7"/>
       <c r="C131" s="7"/>
       <c r="D131" s="7"/>
       <c r="E131" s="7"/>
@@ -3780,7 +3783,7 @@
     </row>
     <row r="132" spans="1:18" ht="14.4" customHeight="1">
       <c r="A132" s="6"/>
-      <c r="B132" s="16"/>
+      <c r="B132" s="7"/>
       <c r="C132" s="7"/>
       <c r="D132" s="7"/>
       <c r="E132" s="7"/>
@@ -3799,7 +3802,7 @@
     </row>
     <row r="133" spans="1:18" ht="14.4" customHeight="1">
       <c r="A133" s="6"/>
-      <c r="B133" s="16"/>
+      <c r="B133" s="7"/>
       <c r="C133" s="7"/>
       <c r="D133" s="7"/>
       <c r="E133" s="7"/>
@@ -3818,7 +3821,7 @@
     </row>
     <row r="134" spans="1:18" ht="14.4" customHeight="1">
       <c r="A134" s="6"/>
-      <c r="B134" s="16"/>
+      <c r="B134" s="7"/>
       <c r="C134" s="7"/>
       <c r="D134" s="7"/>
       <c r="E134" s="7"/>
@@ -3837,7 +3840,7 @@
     </row>
     <row r="135" spans="1:18" ht="14.4" customHeight="1">
       <c r="A135" s="6"/>
-      <c r="B135" s="16"/>
+      <c r="B135" s="7"/>
       <c r="C135" s="7"/>
       <c r="D135" s="7"/>
       <c r="E135" s="7"/>
@@ -3856,7 +3859,7 @@
     </row>
     <row r="136" spans="1:18" ht="14.4" customHeight="1">
       <c r="A136" s="6"/>
-      <c r="B136" s="16"/>
+      <c r="B136" s="7"/>
       <c r="C136" s="7"/>
       <c r="D136" s="7"/>
       <c r="E136" s="7"/>
@@ -3875,7 +3878,7 @@
     </row>
     <row r="137" spans="1:18" ht="14.4" customHeight="1">
       <c r="A137" s="6"/>
-      <c r="B137" s="16"/>
+      <c r="B137" s="7"/>
       <c r="C137" s="7"/>
       <c r="D137" s="7"/>
       <c r="E137" s="7"/>
@@ -3894,7 +3897,7 @@
     </row>
     <row r="138" spans="1:18" ht="14.4" customHeight="1">
       <c r="A138" s="6"/>
-      <c r="B138" s="16"/>
+      <c r="B138" s="7"/>
       <c r="C138" s="7"/>
       <c r="D138" s="7"/>
       <c r="E138" s="7"/>
@@ -3913,7 +3916,7 @@
     </row>
     <row r="139" spans="1:18" ht="14.4" customHeight="1">
       <c r="A139" s="6"/>
-      <c r="B139" s="16"/>
+      <c r="B139" s="7"/>
       <c r="C139" s="7"/>
       <c r="D139" s="7"/>
       <c r="E139" s="7"/>
@@ -3932,7 +3935,7 @@
     </row>
     <row r="140" spans="1:18" ht="14.4" customHeight="1">
       <c r="A140" s="6"/>
-      <c r="B140" s="16"/>
+      <c r="B140" s="7"/>
       <c r="C140" s="7"/>
       <c r="D140" s="7"/>
       <c r="E140" s="7"/>
@@ -3951,7 +3954,7 @@
     </row>
     <row r="141" spans="1:18" ht="14.4" customHeight="1">
       <c r="A141" s="6"/>
-      <c r="B141" s="16"/>
+      <c r="B141" s="7"/>
       <c r="C141" s="7"/>
       <c r="D141" s="7"/>
       <c r="E141" s="7"/>
@@ -3970,7 +3973,7 @@
     </row>
     <row r="142" spans="1:18" ht="14.4" customHeight="1">
       <c r="A142" s="6"/>
-      <c r="B142" s="16"/>
+      <c r="B142" s="7"/>
       <c r="C142" s="7"/>
       <c r="D142" s="7"/>
       <c r="E142" s="7"/>
@@ -3989,7 +3992,7 @@
     </row>
     <row r="143" spans="1:18" ht="14.4" customHeight="1">
       <c r="A143" s="6"/>
-      <c r="B143" s="16"/>
+      <c r="B143" s="7"/>
       <c r="C143" s="7"/>
       <c r="D143" s="7"/>
       <c r="E143" s="7"/>
@@ -4008,7 +4011,7 @@
     </row>
     <row r="144" spans="1:18" ht="14.4" customHeight="1">
       <c r="A144" s="6"/>
-      <c r="B144" s="16"/>
+      <c r="B144" s="7"/>
       <c r="C144" s="7"/>
       <c r="D144" s="7"/>
       <c r="E144" s="7"/>
@@ -4027,7 +4030,7 @@
     </row>
     <row r="145" spans="1:18" ht="14.4" customHeight="1">
       <c r="A145" s="6"/>
-      <c r="B145" s="16"/>
+      <c r="B145" s="7"/>
       <c r="C145" s="7"/>
       <c r="D145" s="7"/>
       <c r="E145" s="7"/>
@@ -4046,7 +4049,7 @@
     </row>
     <row r="146" spans="1:18" ht="14.4" customHeight="1">
       <c r="A146" s="6"/>
-      <c r="B146" s="16"/>
+      <c r="B146" s="7"/>
       <c r="C146" s="7"/>
       <c r="D146" s="7"/>
       <c r="E146" s="7"/>
@@ -4065,7 +4068,7 @@
     </row>
     <row r="147" spans="1:18" ht="14.4" customHeight="1">
       <c r="A147" s="6"/>
-      <c r="B147" s="16"/>
+      <c r="B147" s="7"/>
       <c r="C147" s="7"/>
       <c r="D147" s="7"/>
       <c r="E147" s="7"/>
@@ -4084,7 +4087,7 @@
     </row>
     <row r="148" spans="1:18" ht="14.4" customHeight="1">
       <c r="A148" s="6"/>
-      <c r="B148" s="16"/>
+      <c r="B148" s="7"/>
       <c r="C148" s="7"/>
       <c r="D148" s="7"/>
       <c r="E148" s="7"/>
@@ -4103,7 +4106,7 @@
     </row>
     <row r="149" spans="1:18" ht="14.4" customHeight="1">
       <c r="A149" s="6"/>
-      <c r="B149" s="16"/>
+      <c r="B149" s="7"/>
       <c r="C149" s="7"/>
       <c r="D149" s="7"/>
       <c r="E149" s="7"/>
@@ -4122,7 +4125,7 @@
     </row>
     <row r="150" spans="1:18" ht="14.4" customHeight="1">
       <c r="A150" s="6"/>
-      <c r="B150" s="16"/>
+      <c r="B150" s="7"/>
       <c r="C150" s="7"/>
       <c r="D150" s="7"/>
       <c r="E150" s="7"/>
@@ -4141,7 +4144,7 @@
     </row>
     <row r="151" spans="1:18" ht="14.4" customHeight="1">
       <c r="A151" s="6"/>
-      <c r="B151" s="16"/>
+      <c r="B151" s="7"/>
       <c r="C151" s="7"/>
       <c r="D151" s="7"/>
       <c r="E151" s="7"/>
@@ -4160,7 +4163,7 @@
     </row>
     <row r="152" spans="1:18" ht="14.4" customHeight="1">
       <c r="A152" s="6"/>
-      <c r="B152" s="16"/>
+      <c r="B152" s="7"/>
       <c r="C152" s="7"/>
       <c r="D152" s="7"/>
       <c r="E152" s="7"/>
@@ -4179,7 +4182,7 @@
     </row>
     <row r="153" spans="1:18" ht="14.4" customHeight="1">
       <c r="A153" s="6"/>
-      <c r="B153" s="16"/>
+      <c r="B153" s="7"/>
       <c r="C153" s="7"/>
       <c r="D153" s="7"/>
       <c r="E153" s="7"/>
@@ -4198,7 +4201,7 @@
     </row>
     <row r="154" spans="1:18" ht="14.4" customHeight="1">
       <c r="A154" s="6"/>
-      <c r="B154" s="16"/>
+      <c r="B154" s="7"/>
       <c r="C154" s="7"/>
       <c r="D154" s="7"/>
       <c r="E154" s="7"/>
@@ -4217,7 +4220,7 @@
     </row>
     <row r="155" spans="1:18" ht="14.4" customHeight="1">
       <c r="A155" s="6"/>
-      <c r="B155" s="16"/>
+      <c r="B155" s="7"/>
       <c r="C155" s="7"/>
       <c r="D155" s="7"/>
       <c r="E155" s="7"/>
@@ -4236,7 +4239,7 @@
     </row>
     <row r="156" spans="1:18" ht="14.4" customHeight="1">
       <c r="A156" s="6"/>
-      <c r="B156" s="16"/>
+      <c r="B156" s="7"/>
       <c r="C156" s="7"/>
       <c r="D156" s="7"/>
       <c r="E156" s="7"/>
@@ -4255,7 +4258,7 @@
     </row>
     <row r="157" spans="1:18" ht="14.4" customHeight="1">
       <c r="A157" s="6"/>
-      <c r="B157" s="16"/>
+      <c r="B157" s="7"/>
       <c r="C157" s="7"/>
       <c r="D157" s="7"/>
       <c r="E157" s="7"/>
@@ -4274,7 +4277,7 @@
     </row>
     <row r="158" spans="1:18" ht="14.4" customHeight="1">
       <c r="A158" s="6"/>
-      <c r="B158" s="16"/>
+      <c r="B158" s="7"/>
       <c r="C158" s="7"/>
       <c r="D158" s="7"/>
       <c r="E158" s="7"/>
@@ -4293,7 +4296,7 @@
     </row>
     <row r="159" spans="1:18" ht="14.4" customHeight="1">
       <c r="A159" s="6"/>
-      <c r="B159" s="16"/>
+      <c r="B159" s="7"/>
       <c r="C159" s="7"/>
       <c r="D159" s="7"/>
       <c r="E159" s="7"/>
@@ -4312,7 +4315,7 @@
     </row>
     <row r="160" spans="1:18" ht="14.4" customHeight="1">
       <c r="A160" s="6"/>
-      <c r="B160" s="16"/>
+      <c r="B160" s="7"/>
       <c r="C160" s="7"/>
       <c r="D160" s="7"/>
       <c r="E160" s="7"/>
@@ -4331,7 +4334,7 @@
     </row>
     <row r="161" spans="1:18" ht="14.4" customHeight="1">
       <c r="A161" s="6"/>
-      <c r="B161" s="16"/>
+      <c r="B161" s="7"/>
       <c r="C161" s="7"/>
       <c r="D161" s="7"/>
       <c r="E161" s="7"/>
@@ -4350,7 +4353,7 @@
     </row>
     <row r="162" spans="1:18" ht="14.4" customHeight="1">
       <c r="A162" s="6"/>
-      <c r="B162" s="16"/>
+      <c r="B162" s="7"/>
       <c r="C162" s="7"/>
       <c r="D162" s="7"/>
       <c r="E162" s="7"/>
@@ -4369,7 +4372,7 @@
     </row>
     <row r="163" spans="1:18" ht="14.4" customHeight="1">
       <c r="A163" s="6"/>
-      <c r="B163" s="16"/>
+      <c r="B163" s="7"/>
       <c r="C163" s="7"/>
       <c r="D163" s="7"/>
       <c r="E163" s="7"/>
@@ -4388,7 +4391,7 @@
     </row>
     <row r="164" spans="1:18" ht="14.4" customHeight="1">
       <c r="A164" s="6"/>
-      <c r="B164" s="16"/>
+      <c r="B164" s="7"/>
       <c r="C164" s="7"/>
       <c r="D164" s="7"/>
       <c r="E164" s="7"/>
@@ -4407,7 +4410,7 @@
     </row>
     <row r="165" spans="1:18" ht="14.4" customHeight="1">
       <c r="A165" s="6"/>
-      <c r="B165" s="16"/>
+      <c r="B165" s="7"/>
       <c r="C165" s="7"/>
       <c r="D165" s="7"/>
       <c r="E165" s="7"/>
@@ -4426,7 +4429,7 @@
     </row>
     <row r="166" spans="1:18" ht="14.4" customHeight="1">
       <c r="A166" s="6"/>
-      <c r="B166" s="16"/>
+      <c r="B166" s="7"/>
       <c r="C166" s="7"/>
       <c r="D166" s="7"/>
       <c r="E166" s="7"/>
@@ -4445,7 +4448,7 @@
     </row>
     <row r="167" spans="1:18" ht="14.4" customHeight="1">
       <c r="A167" s="6"/>
-      <c r="B167" s="16"/>
+      <c r="B167" s="7"/>
       <c r="C167" s="7"/>
       <c r="D167" s="7"/>
       <c r="E167" s="7"/>
@@ -4464,7 +4467,7 @@
     </row>
     <row r="168" spans="1:18" ht="14.4" customHeight="1">
       <c r="A168" s="6"/>
-      <c r="B168" s="16"/>
+      <c r="B168" s="7"/>
       <c r="C168" s="7"/>
       <c r="D168" s="7"/>
       <c r="E168" s="7"/>
@@ -4483,7 +4486,7 @@
     </row>
     <row r="169" spans="1:18" ht="14.4" customHeight="1">
       <c r="A169" s="6"/>
-      <c r="B169" s="16"/>
+      <c r="B169" s="7"/>
       <c r="C169" s="7"/>
       <c r="D169" s="7"/>
       <c r="E169" s="7"/>
@@ -4502,7 +4505,7 @@
     </row>
     <row r="170" spans="1:18" ht="14.4" customHeight="1">
       <c r="A170" s="6"/>
-      <c r="B170" s="16"/>
+      <c r="B170" s="7"/>
       <c r="C170" s="7"/>
       <c r="D170" s="7"/>
       <c r="E170" s="7"/>
@@ -4521,7 +4524,7 @@
     </row>
     <row r="171" spans="1:18" ht="14.4" customHeight="1">
       <c r="A171" s="6"/>
-      <c r="B171" s="16"/>
+      <c r="B171" s="7"/>
       <c r="C171" s="7"/>
       <c r="D171" s="7"/>
       <c r="E171" s="7"/>
@@ -4540,7 +4543,7 @@
     </row>
     <row r="172" spans="1:18" ht="14.4" customHeight="1">
       <c r="A172" s="6"/>
-      <c r="B172" s="16"/>
+      <c r="B172" s="7"/>
       <c r="C172" s="7"/>
       <c r="D172" s="7"/>
       <c r="E172" s="7"/>
@@ -4559,7 +4562,7 @@
     </row>
     <row r="173" spans="1:18" ht="14.4" customHeight="1">
       <c r="A173" s="6"/>
-      <c r="B173" s="16"/>
+      <c r="B173" s="7"/>
       <c r="C173" s="7"/>
       <c r="D173" s="7"/>
       <c r="E173" s="7"/>
@@ -4578,7 +4581,7 @@
     </row>
     <row r="174" spans="1:18" ht="14.4" customHeight="1">
       <c r="A174" s="6"/>
-      <c r="B174" s="16"/>
+      <c r="B174" s="7"/>
       <c r="C174" s="7"/>
       <c r="D174" s="7"/>
       <c r="E174" s="7"/>
@@ -4597,7 +4600,7 @@
     </row>
     <row r="175" spans="1:18" ht="14.4" customHeight="1">
       <c r="A175" s="6"/>
-      <c r="B175" s="16"/>
+      <c r="B175" s="7"/>
       <c r="C175" s="7"/>
       <c r="D175" s="7"/>
       <c r="E175" s="7"/>
@@ -4616,7 +4619,7 @@
     </row>
     <row r="176" spans="1:18" ht="14.4" customHeight="1">
       <c r="A176" s="6"/>
-      <c r="B176" s="16"/>
+      <c r="B176" s="7"/>
       <c r="C176" s="7"/>
       <c r="D176" s="7"/>
       <c r="E176" s="7"/>
@@ -4635,7 +4638,7 @@
     </row>
     <row r="177" spans="1:18" ht="14.4" customHeight="1">
       <c r="A177" s="6"/>
-      <c r="B177" s="16"/>
+      <c r="B177" s="7"/>
       <c r="C177" s="7"/>
       <c r="D177" s="7"/>
       <c r="E177" s="7"/>
@@ -4654,7 +4657,7 @@
     </row>
     <row r="178" spans="1:18" ht="14.4" customHeight="1">
       <c r="A178" s="6"/>
-      <c r="B178" s="16"/>
+      <c r="B178" s="7"/>
       <c r="C178" s="7"/>
       <c r="D178" s="7"/>
       <c r="E178" s="7"/>
@@ -4673,7 +4676,7 @@
     </row>
     <row r="179" spans="1:18" ht="14.4" customHeight="1">
       <c r="A179" s="6"/>
-      <c r="B179" s="16"/>
+      <c r="B179" s="7"/>
       <c r="C179" s="7"/>
       <c r="D179" s="7"/>
       <c r="E179" s="7"/>
@@ -4692,7 +4695,7 @@
     </row>
     <row r="180" spans="1:18" ht="14.4" customHeight="1">
       <c r="A180" s="6"/>
-      <c r="B180" s="16"/>
+      <c r="B180" s="7"/>
       <c r="C180" s="7"/>
       <c r="D180" s="7"/>
       <c r="E180" s="7"/>
@@ -4711,7 +4714,7 @@
     </row>
     <row r="181" spans="1:18" ht="14.4" customHeight="1">
       <c r="A181" s="6"/>
-      <c r="B181" s="16"/>
+      <c r="B181" s="7"/>
       <c r="C181" s="7"/>
       <c r="D181" s="7"/>
       <c r="E181" s="7"/>
@@ -4730,7 +4733,7 @@
     </row>
     <row r="182" spans="1:18" ht="14.4" customHeight="1">
       <c r="A182" s="6"/>
-      <c r="B182" s="16"/>
+      <c r="B182" s="7"/>
       <c r="C182" s="7"/>
       <c r="D182" s="7"/>
       <c r="E182" s="7"/>
@@ -4749,7 +4752,7 @@
     </row>
     <row r="183" spans="1:18" ht="14.4" customHeight="1">
       <c r="A183" s="6"/>
-      <c r="B183" s="16"/>
+      <c r="B183" s="7"/>
       <c r="C183" s="7"/>
       <c r="D183" s="7"/>
       <c r="E183" s="7"/>
@@ -4768,7 +4771,7 @@
     </row>
     <row r="184" spans="1:18" ht="14.4" customHeight="1">
       <c r="A184" s="6"/>
-      <c r="B184" s="16"/>
+      <c r="B184" s="7"/>
       <c r="C184" s="7"/>
       <c r="D184" s="7"/>
       <c r="E184" s="7"/>
@@ -4787,7 +4790,7 @@
     </row>
     <row r="185" spans="1:18" ht="14.4" customHeight="1">
       <c r="A185" s="6"/>
-      <c r="B185" s="16"/>
+      <c r="B185" s="7"/>
       <c r="C185" s="7"/>
       <c r="D185" s="7"/>
       <c r="E185" s="7"/>
@@ -4806,7 +4809,7 @@
     </row>
     <row r="186" spans="1:18" ht="14.4" customHeight="1">
       <c r="A186" s="6"/>
-      <c r="B186" s="16"/>
+      <c r="B186" s="7"/>
       <c r="C186" s="7"/>
       <c r="D186" s="7"/>
       <c r="E186" s="7"/>
@@ -4825,7 +4828,7 @@
     </row>
     <row r="187" spans="1:18" ht="14.4" customHeight="1">
       <c r="A187" s="6"/>
-      <c r="B187" s="16"/>
+      <c r="B187" s="7"/>
       <c r="C187" s="7"/>
       <c r="D187" s="7"/>
       <c r="E187" s="7"/>
@@ -4844,7 +4847,7 @@
     </row>
     <row r="188" spans="1:18" ht="14.4" customHeight="1">
       <c r="A188" s="6"/>
-      <c r="B188" s="16"/>
+      <c r="B188" s="7"/>
       <c r="C188" s="7"/>
       <c r="D188" s="7"/>
       <c r="E188" s="7"/>
@@ -4863,7 +4866,7 @@
     </row>
     <row r="189" spans="1:18" ht="14.4" customHeight="1">
       <c r="A189" s="6"/>
-      <c r="B189" s="16"/>
+      <c r="B189" s="7"/>
       <c r="C189" s="7"/>
       <c r="D189" s="7"/>
       <c r="E189" s="7"/>
@@ -4882,7 +4885,7 @@
     </row>
     <row r="190" spans="1:18" ht="14.4" customHeight="1">
       <c r="A190" s="6"/>
-      <c r="B190" s="16"/>
+      <c r="B190" s="7"/>
       <c r="C190" s="7"/>
       <c r="D190" s="7"/>
       <c r="E190" s="7"/>
@@ -4901,7 +4904,7 @@
     </row>
     <row r="191" spans="1:18" ht="14.4" customHeight="1">
       <c r="A191" s="6"/>
-      <c r="B191" s="16"/>
+      <c r="B191" s="7"/>
       <c r="C191" s="7"/>
       <c r="D191" s="7"/>
       <c r="E191" s="7"/>
@@ -4920,7 +4923,7 @@
     </row>
     <row r="192" spans="1:18" ht="14.4" customHeight="1">
       <c r="A192" s="6"/>
-      <c r="B192" s="16"/>
+      <c r="B192" s="7"/>
       <c r="C192" s="7"/>
       <c r="D192" s="7"/>
       <c r="E192" s="7"/>
@@ -4939,7 +4942,7 @@
     </row>
     <row r="193" spans="1:18" ht="14.4" customHeight="1">
       <c r="A193" s="6"/>
-      <c r="B193" s="16"/>
+      <c r="B193" s="7"/>
       <c r="C193" s="7"/>
       <c r="D193" s="7"/>
       <c r="E193" s="7"/>
@@ -4958,7 +4961,7 @@
     </row>
     <row r="194" spans="1:18" ht="14.4" customHeight="1">
       <c r="A194" s="6"/>
-      <c r="B194" s="16"/>
+      <c r="B194" s="7"/>
       <c r="C194" s="7"/>
       <c r="D194" s="7"/>
       <c r="E194" s="7"/>
@@ -4977,7 +4980,7 @@
     </row>
     <row r="195" spans="1:18" ht="14.4" customHeight="1">
       <c r="A195" s="6"/>
-      <c r="B195" s="16"/>
+      <c r="B195" s="7"/>
       <c r="C195" s="7"/>
       <c r="D195" s="7"/>
       <c r="E195" s="7"/>
@@ -4996,7 +4999,7 @@
     </row>
     <row r="196" spans="1:18" ht="14.4" customHeight="1">
       <c r="A196" s="6"/>
-      <c r="B196" s="16"/>
+      <c r="B196" s="7"/>
       <c r="C196" s="7"/>
       <c r="D196" s="7"/>
       <c r="E196" s="7"/>
@@ -5015,7 +5018,7 @@
     </row>
     <row r="197" spans="1:18" ht="14.4" customHeight="1">
       <c r="A197" s="6"/>
-      <c r="B197" s="16"/>
+      <c r="B197" s="7"/>
       <c r="C197" s="7"/>
       <c r="D197" s="7"/>
       <c r="E197" s="7"/>
@@ -5034,7 +5037,7 @@
     </row>
     <row r="198" spans="1:18" ht="14.4" customHeight="1">
       <c r="A198" s="6"/>
-      <c r="B198" s="16"/>
+      <c r="B198" s="7"/>
       <c r="C198" s="7"/>
       <c r="D198" s="7"/>
       <c r="E198" s="7"/>
@@ -5053,7 +5056,7 @@
     </row>
     <row r="199" spans="1:18" ht="14.4" customHeight="1">
       <c r="A199" s="6"/>
-      <c r="B199" s="16"/>
+      <c r="B199" s="7"/>
       <c r="C199" s="7"/>
       <c r="D199" s="7"/>
       <c r="E199" s="7"/>
@@ -5091,284 +5094,279 @@
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="G3:I8 A9:I199 A3:D8">
-    <cfRule type="expression" dxfId="64" priority="15">
+  <conditionalFormatting sqref="A3:D8 G3:I8 A9:I199">
+    <cfRule type="expression" dxfId="63" priority="15">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="16">
+    <cfRule type="expression" dxfId="62" priority="16">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:I8 A2:I2 A9:I200 A3:D8">
-    <cfRule type="expression" dxfId="62" priority="78">
+  <conditionalFormatting sqref="A2:I2 A3:D8 G3:I8 A9:I200">
+    <cfRule type="expression" dxfId="61" priority="78">
       <formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:I8 A2:I2 A9:I200 A3:D8">
-    <cfRule type="expression" dxfId="61" priority="77">
+  <conditionalFormatting sqref="A2:I2 G3:I8 A9:I200 A3:D8">
+    <cfRule type="expression" dxfId="60" priority="77">
       <formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:C8">
-    <cfRule type="expression" dxfId="60" priority="191">
+    <cfRule type="expression" dxfId="59" priority="191">
       <formula>#REF!&gt;#REF!</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="192">
+    <cfRule type="expression" dxfId="58" priority="192">
       <formula>AND($A3&lt;&gt;"",#REF!&gt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D199">
-    <cfRule type="expression" dxfId="58" priority="17">
+    <cfRule type="expression" dxfId="57" priority="17">
       <formula>$D6&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="expression" dxfId="57" priority="19">
+    <cfRule type="expression" dxfId="56" priority="19">
       <formula>$E2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E8">
-    <cfRule type="expression" dxfId="56" priority="6">
+    <cfRule type="expression" dxfId="55" priority="6">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="7">
+    <cfRule type="expression" dxfId="54" priority="7">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:F199">
-    <cfRule type="expression" dxfId="54" priority="8">
+    <cfRule type="expression" dxfId="53" priority="8">
       <formula>$E9&gt;$F9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2">
-    <cfRule type="expression" dxfId="53" priority="30">
+    <cfRule type="expression" dxfId="52" priority="30">
       <formula>$F2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F8">
-    <cfRule type="expression" dxfId="52" priority="4">
+    <cfRule type="expression" dxfId="51" priority="4">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="5">
+    <cfRule type="expression" dxfId="50" priority="5">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9:F199">
+    <cfRule type="expression" dxfId="49" priority="213">
+      <formula>AND($A9&lt;&gt;"",$F9&gt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G3">
-    <cfRule type="expression" dxfId="50" priority="33">
+    <cfRule type="expression" dxfId="48" priority="33">
       <formula>$G2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4:I8 G3:L3 A9:I199 A3:D8">
-    <cfRule type="expression" dxfId="49" priority="13">
+  <conditionalFormatting sqref="G3">
+    <cfRule type="expression" dxfId="47" priority="214">
+      <formula>AND($A3&lt;&gt;"",#REF!&gt;$G3)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="46" priority="215">
+      <formula>AND($A3&lt;&gt;"",$G3&gt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G199">
+    <cfRule type="expression" dxfId="45" priority="216">
+      <formula>AND($A4&lt;&gt;"",OR($F4="",#REF!=""))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="217">
+      <formula>#REF!&gt;$G4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:H199">
+    <cfRule type="expression" dxfId="43" priority="23">
+      <formula>AND($A4&lt;&gt;"",$G4&gt;$H4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:I8 A9:I199 G3:L3 A3:D8">
+    <cfRule type="expression" dxfId="42" priority="13">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:L3 G4:I8 A9:I199 A3:D8">
-    <cfRule type="expression" dxfId="48" priority="14">
+  <conditionalFormatting sqref="G3:L3 A3:D8 G4:I8 A9:I199">
+    <cfRule type="expression" dxfId="41" priority="14">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="expression" dxfId="47" priority="35">
+    <cfRule type="expression" dxfId="40" priority="35">
       <formula>$H2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4:H199">
-    <cfRule type="expression" dxfId="46" priority="23">
-      <formula>AND($A4&lt;&gt;"",$G4&gt;$H4)</formula>
+  <conditionalFormatting sqref="H3 H4:I199">
+    <cfRule type="expression" dxfId="39" priority="227">
+      <formula>AND($A3&lt;&gt;"",$H3&gt;$I3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" dxfId="38" priority="140">
+      <formula>AND($A3&lt;&gt;"",#REF!&gt;$H3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:I199">
-    <cfRule type="expression" dxfId="45" priority="9">
+    <cfRule type="expression" dxfId="37" priority="9">
       <formula>$H4&gt;$I4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I3">
-    <cfRule type="expression" dxfId="44" priority="37">
+    <cfRule type="expression" dxfId="36" priority="37">
       <formula>$I2&gt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3">
-    <cfRule type="expression" dxfId="43" priority="140">
-      <formula>AND($A3&lt;&gt;"",#REF!&gt;$H3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="42" priority="183">
+    <cfRule type="expression" dxfId="35" priority="183">
       <formula>AND($A3&lt;&gt;"",#REF!&gt;$I3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I199">
+    <cfRule type="expression" dxfId="34" priority="231">
+      <formula>AND($A3&lt;&gt;"",$I3&gt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J200">
+    <cfRule type="expression" dxfId="33" priority="232">
+      <formula>AND($A3&lt;&gt;"",#REF!&gt;$J3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J200">
-    <cfRule type="expression" dxfId="41" priority="88">
+    <cfRule type="expression" dxfId="32" priority="88">
       <formula>#REF!&gt;$J5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J4:K4">
-    <cfRule type="expression" dxfId="40" priority="61">
+    <cfRule type="expression" dxfId="31" priority="61">
       <formula>AND(#REF!&lt;&gt;"",$J4&gt;$K4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:K7 J8:J10 J11:K200">
+    <cfRule type="expression" dxfId="30" priority="102">
+      <formula>AND($A4&lt;&gt;"",$J5&gt;$K5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J4:O4">
-    <cfRule type="expression" dxfId="39" priority="52">
+    <cfRule type="expression" dxfId="29" priority="52">
       <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="53">
+    <cfRule type="expression" dxfId="28" priority="53">
       <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:O7 J8:J10 L8:O10 J11:O200">
-    <cfRule type="expression" dxfId="37" priority="51">
+    <cfRule type="expression" dxfId="27" priority="51">
       <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:O7 L8:O10 J11:O200 J8:J10">
-    <cfRule type="expression" dxfId="36" priority="50">
+    <cfRule type="expression" dxfId="26" priority="50">
       <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J4:R4">
-    <cfRule type="expression" dxfId="35" priority="56">
+    <cfRule type="expression" dxfId="25" priority="56">
       <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="57">
+    <cfRule type="expression" dxfId="24" priority="57">
       <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:R7 J8:J10 L8:R10 J11:R200">
-    <cfRule type="expression" dxfId="33" priority="54">
+    <cfRule type="expression" dxfId="23" priority="55">
+      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="54">
       <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="55">
-      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:K10">
+    <cfRule type="expression" dxfId="21" priority="236">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="237">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="238">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="239">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="17" priority="240">
+      <formula>$K9&gt;$L8</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="241">
+      <formula>AND($A7&lt;&gt;"",$J8&gt;$K9)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="242">
+      <formula>AND($A7&lt;&gt;"",$K9&gt;$L8)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:L3">
+    <cfRule type="expression" dxfId="14" priority="243">
+      <formula>AND($A3&lt;&gt;"",$K3&gt;$L3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4:L4">
-    <cfRule type="expression" dxfId="31" priority="64">
+    <cfRule type="expression" dxfId="13" priority="64">
       <formula>AND(#REF!&lt;&gt;"",$K4&gt;$L4)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4:L7 L8:L10 K11:L200">
-    <cfRule type="expression" dxfId="30" priority="11">
+    <cfRule type="expression" dxfId="12" priority="11">
       <formula>$K4&gt;$L4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:K7 J8:J10 J11:K200">
-    <cfRule type="expression" dxfId="29" priority="102">
-      <formula>AND($A4&lt;&gt;"",$J5&gt;$K5)</formula>
+  <conditionalFormatting sqref="K5:L7 L8:L10 K11:L200">
+    <cfRule type="expression" dxfId="11" priority="62">
+      <formula>AND($A4&lt;&gt;"",$K5&gt;$L5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4:M4">
-    <cfRule type="expression" dxfId="28" priority="65">
+    <cfRule type="expression" dxfId="10" priority="65">
       <formula>AND(#REF!&lt;&gt;"",$L4&gt;$M4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L7 L8:L10 K11:L200">
-    <cfRule type="expression" dxfId="27" priority="62">
-      <formula>AND($A4&lt;&gt;"",$K5&gt;$L5)</formula>
+  <conditionalFormatting sqref="L5:M200">
+    <cfRule type="expression" dxfId="9" priority="63">
+      <formula>AND($A4&lt;&gt;"",$L5&gt;$M5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4:N4">
-    <cfRule type="expression" dxfId="26" priority="67">
+    <cfRule type="expression" dxfId="8" priority="67">
       <formula>AND(#REF!&lt;&gt;"",$M4&gt;$N4)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4:N6">
-    <cfRule type="expression" dxfId="25" priority="12">
+    <cfRule type="expression" dxfId="7" priority="12">
       <formula>$M4&gt;$N4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5:M200">
-    <cfRule type="expression" dxfId="24" priority="63">
-      <formula>AND($A4&lt;&gt;"",$L5&gt;$M5)</formula>
+  <conditionalFormatting sqref="M5:N200">
+    <cfRule type="expression" dxfId="6" priority="66">
+      <formula>AND($A4&lt;&gt;"",$M5&gt;$N5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:O4">
-    <cfRule type="expression" dxfId="23" priority="69">
+    <cfRule type="expression" dxfId="5" priority="69">
       <formula>AND(#REF!&lt;&gt;"",$N4&gt;$O4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:N200">
-    <cfRule type="expression" dxfId="22" priority="66">
-      <formula>AND($A4&lt;&gt;"",$M5&gt;$N5)</formula>
+  <conditionalFormatting sqref="N5:O200">
+    <cfRule type="expression" dxfId="4" priority="68">
+      <formula>AND($A4&lt;&gt;"",$N5&gt;$O5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O4:P4">
-    <cfRule type="expression" dxfId="21" priority="71">
+    <cfRule type="expression" dxfId="3" priority="71">
       <formula>AND(#REF!&lt;&gt;"",$O4&gt;$P4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N5:O200">
-    <cfRule type="expression" dxfId="20" priority="68">
-      <formula>AND($A4&lt;&gt;"",$N5&gt;$O5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q4:R4">
-    <cfRule type="expression" dxfId="19" priority="73">
-      <formula>AND(#REF!&lt;&gt;"",$Q4&gt;$R4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F199">
-    <cfRule type="expression" dxfId="18" priority="213">
-      <formula>AND($A9&lt;&gt;"",$F9&gt;#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="17" priority="214">
-      <formula>AND($A3&lt;&gt;"",#REF!&gt;$G3)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="215">
-      <formula>AND($A3&lt;&gt;"",$G3&gt;#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:G199">
-    <cfRule type="expression" dxfId="15" priority="216">
-      <formula>AND($A4&lt;&gt;"",OR($F4="",#REF!=""))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="217">
-      <formula>#REF!&gt;$G4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3 H4:I199">
-    <cfRule type="expression" dxfId="13" priority="227">
-      <formula>AND($A3&lt;&gt;"",$H3&gt;$I3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I199">
-    <cfRule type="expression" dxfId="12" priority="231">
-      <formula>AND($A3&lt;&gt;"",$I3&gt;#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3:J200">
-    <cfRule type="expression" dxfId="11" priority="232">
-      <formula>AND($A3&lt;&gt;"",#REF!&gt;$J3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K9:K10">
-    <cfRule type="expression" dxfId="10" priority="236">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="237">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="238">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="239">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="240">
-      <formula>$K9&gt;$L8</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="241">
-      <formula>AND($A7&lt;&gt;"",$J8&gt;$K9)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="242">
-      <formula>AND($A7&lt;&gt;"",$K9&gt;$L8)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3:L3">
-    <cfRule type="expression" dxfId="3" priority="243">
-      <formula>AND($A3&lt;&gt;"",$K3&gt;$L3)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:P200">
@@ -5376,8 +5374,13 @@
       <formula>AND($A4&lt;&gt;"",$O5&gt;$P5)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q4:R4">
+    <cfRule type="expression" dxfId="1" priority="73">
+      <formula>AND(#REF!&lt;&gt;"",$Q4&gt;$R4)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="Q5:R200">
-    <cfRule type="expression" dxfId="1" priority="253">
+    <cfRule type="expression" dxfId="0" priority="253">
       <formula>AND($A4&lt;&gt;"",$Q5&gt;$R5)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat : conversation 기능 추가
</commit_message>
<xml_diff>
--- a/Assets/Excels/CreatureData.xlsx
+++ b/Assets/Excels/CreatureData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devs\TRPG.Client\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78313D57-3971-460B-B56D-BB8D6B467B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{893AFF55-3B2E-4798-9FB2-1AAB06D83BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreatureData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>Id</t>
   </si>
@@ -139,6 +139,18 @@
   </si>
   <si>
     <t>Monster_05</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster_000</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>PF_Cheshire</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>체셔</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -382,7 +394,217 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="86">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -993,7 +1215,7 @@
   <autoFilter ref="A1:I200" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
-    <tableColumn id="8" xr3:uid="{FC26B9EF-D3B9-43E3-BEBA-CBD0BF0F99C1}" name="PfId" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{FC26B9EF-D3B9-43E3-BEBA-CBD0BF0F99C1}" name="PfId" dataDxfId="85"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Description"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DisplayName"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Type"/>
@@ -1228,19 +1450,19 @@
     </row>
     <row r="3" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A3" s="6" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>12</v>
@@ -1262,19 +1484,19 @@
     </row>
     <row r="4" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A4" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>13</v>
+      <c r="D4" s="15" t="s">
+        <v>10</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>12</v>
@@ -1299,19 +1521,19 @@
     </row>
     <row r="5" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A5" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>12</v>
@@ -1336,19 +1558,19 @@
     </row>
     <row r="6" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A6" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>20</v>
+      <c r="D6" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="14" t="s">
         <v>12</v>
@@ -1373,19 +1595,19 @@
     </row>
     <row r="7" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A7" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>12</v>
@@ -1410,19 +1632,19 @@
     </row>
     <row r="8" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A8" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>12</v>
@@ -1444,16 +1666,34 @@
       <c r="Q8"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18" ht="14.4" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
+    <row r="9" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
+      <c r="A9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="8">
+        <v>10</v>
+      </c>
+      <c r="H9" s="8">
+        <v>10</v>
+      </c>
+      <c r="I9" s="8">
+        <v>10</v>
+      </c>
       <c r="J9" s="9"/>
       <c r="K9" s="9"/>
       <c r="L9" s="9"/>
@@ -1463,13 +1703,13 @@
       <c r="Q9"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18" ht="14.4" customHeight="1">
+    <row r="10" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A10" s="6"/>
       <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
+      <c r="C10" s="8"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="8"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
       <c r="I10" s="8"/>
@@ -1482,13 +1722,13 @@
       <c r="Q10"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18" ht="14.4" customHeight="1">
+    <row r="11" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A11" s="6"/>
       <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
+      <c r="C11" s="8"/>
       <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="8"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
       <c r="I11" s="8"/>
@@ -1501,13 +1741,13 @@
       <c r="Q11"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18" ht="14.4" customHeight="1">
+    <row r="12" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -1520,13 +1760,13 @@
       <c r="Q12"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18" ht="14.4" customHeight="1">
+    <row r="13" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A13" s="6"/>
       <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -1539,13 +1779,13 @@
       <c r="Q13"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18" ht="14.4" customHeight="1">
+    <row r="14" spans="1:18" ht="14.4" customHeight="1" thickBot="1">
       <c r="A14" s="6"/>
       <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -5094,301 +5334,382 @@
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
-  <conditionalFormatting sqref="A3:D8 G3:I8 A9:I199">
-    <cfRule type="expression" dxfId="63" priority="15">
+  <conditionalFormatting sqref="A15:I199 A3:D14 G3:I14">
+    <cfRule type="expression" dxfId="84" priority="36">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="16">
+    <cfRule type="expression" dxfId="83" priority="37">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:I2 A3:D8 G3:I8 A9:I200">
-    <cfRule type="expression" dxfId="61" priority="78">
+  <conditionalFormatting sqref="A2:I2 A15:I200 A3:D14 G3:I14">
+    <cfRule type="expression" dxfId="82" priority="99">
       <formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:I2 G3:I8 A9:I200 A3:D8">
-    <cfRule type="expression" dxfId="60" priority="77">
+  <conditionalFormatting sqref="A2:I2 A15:I200 G3:I14 A3:D14">
+    <cfRule type="expression" dxfId="81" priority="98">
       <formula>AND($A2&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C8">
-    <cfRule type="expression" dxfId="59" priority="191">
+  <conditionalFormatting sqref="C3:C14">
+    <cfRule type="expression" dxfId="80" priority="212">
       <formula>#REF!&gt;#REF!</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="192">
+    <cfRule type="expression" dxfId="79" priority="213">
       <formula>AND($A3&lt;&gt;"",#REF!&gt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D199">
-    <cfRule type="expression" dxfId="57" priority="17">
+  <conditionalFormatting sqref="D12:D199 D6:D9">
+    <cfRule type="expression" dxfId="78" priority="38">
       <formula>$D6&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="expression" dxfId="56" priority="19">
+    <cfRule type="expression" dxfId="77" priority="40">
       <formula>$E2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E8">
-    <cfRule type="expression" dxfId="55" priority="6">
+  <conditionalFormatting sqref="E3:E14">
+    <cfRule type="expression" dxfId="76" priority="27">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="7">
+    <cfRule type="expression" dxfId="75" priority="28">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E9:F199">
-    <cfRule type="expression" dxfId="53" priority="8">
-      <formula>$E9&gt;$F9</formula>
+  <conditionalFormatting sqref="E15:F199">
+    <cfRule type="expression" dxfId="74" priority="29">
+      <formula>$E15&gt;$F15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2">
-    <cfRule type="expression" dxfId="52" priority="30">
+    <cfRule type="expression" dxfId="73" priority="51">
       <formula>$F2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F8">
-    <cfRule type="expression" dxfId="51" priority="4">
+  <conditionalFormatting sqref="F3:F14">
+    <cfRule type="expression" dxfId="72" priority="25">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="5">
+    <cfRule type="expression" dxfId="71" priority="26">
       <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F199">
-    <cfRule type="expression" dxfId="49" priority="213">
-      <formula>AND($A9&lt;&gt;"",$F9&gt;#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G3">
-    <cfRule type="expression" dxfId="48" priority="33">
+  <conditionalFormatting sqref="F15:F199">
+    <cfRule type="expression" dxfId="70" priority="234">
+      <formula>AND($A15&lt;&gt;"",$F15&gt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" dxfId="69" priority="54">
       <formula>$G2&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G199">
+    <cfRule type="expression" dxfId="66" priority="237">
+      <formula>AND($A4&lt;&gt;"",OR($F4="",#REF!=""))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="238">
+      <formula>#REF!&gt;$G4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:H199">
+    <cfRule type="expression" dxfId="64" priority="44">
+      <formula>AND($A4&lt;&gt;"",$G4&gt;$H4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15:I199 J3:L3 G3:I14 A3:D14">
+    <cfRule type="expression" dxfId="63" priority="34">
+      <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:L3 A15:I199 A3:D14 G3:I14">
+    <cfRule type="expression" dxfId="62" priority="35">
+      <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2">
+    <cfRule type="expression" dxfId="61" priority="56">
+      <formula>$H2&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3 H4:I199">
+    <cfRule type="expression" dxfId="60" priority="248">
+      <formula>AND($A3&lt;&gt;"",$H3&gt;$I3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4:I199">
+    <cfRule type="expression" dxfId="58" priority="30">
+      <formula>$H4&gt;$I4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2">
+    <cfRule type="expression" dxfId="57" priority="58">
+      <formula>$I2&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:I199">
+    <cfRule type="expression" dxfId="55" priority="252">
+      <formula>AND($A3&lt;&gt;"",$I3&gt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J200">
+    <cfRule type="expression" dxfId="54" priority="253">
+      <formula>AND($A3&lt;&gt;"",#REF!&gt;$J3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J200">
+    <cfRule type="expression" dxfId="53" priority="109">
+      <formula>#REF!&gt;$J5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4:K4">
+    <cfRule type="expression" dxfId="52" priority="82">
+      <formula>AND(#REF!&lt;&gt;"",$J4&gt;$K4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:K7 J8:J10 J11:K200">
+    <cfRule type="expression" dxfId="51" priority="123">
+      <formula>AND($A4&lt;&gt;"",$J5&gt;$K5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4:O4">
+    <cfRule type="expression" dxfId="50" priority="73">
+      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="49" priority="74">
+      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:O7 J8:J10 L8:O10 J11:O200">
+    <cfRule type="expression" dxfId="48" priority="72">
+      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:O7 L8:O10 J11:O200 J8:J10">
+    <cfRule type="expression" dxfId="47" priority="71">
+      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4:R4">
+    <cfRule type="expression" dxfId="46" priority="77">
+      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="78">
+      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:R7 J8:J10 L8:R10 J11:R200">
+    <cfRule type="expression" dxfId="44" priority="76">
+      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="75">
+      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:K10">
+    <cfRule type="expression" dxfId="42" priority="257">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="41" priority="258">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="40" priority="259">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="260">
+      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="261">
+      <formula>$K9&gt;$L8</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="262">
+      <formula>AND($A7&lt;&gt;"",$J8&gt;$K9)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="36" priority="263">
+      <formula>AND($A7&lt;&gt;"",$K9&gt;$L8)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:L3">
+    <cfRule type="expression" dxfId="35" priority="264">
+      <formula>AND($A3&lt;&gt;"",$K3&gt;$L3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4:L4">
+    <cfRule type="expression" dxfId="34" priority="85">
+      <formula>AND(#REF!&lt;&gt;"",$K4&gt;$L4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4:L7 L8:L10 K11:L200">
+    <cfRule type="expression" dxfId="33" priority="32">
+      <formula>$K4&gt;$L4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:L7 L8:L10 K11:L200">
+    <cfRule type="expression" dxfId="32" priority="83">
+      <formula>AND($A4&lt;&gt;"",$K5&gt;$L5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L4:M4">
+    <cfRule type="expression" dxfId="31" priority="86">
+      <formula>AND(#REF!&lt;&gt;"",$L4&gt;$M4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:M200">
+    <cfRule type="expression" dxfId="30" priority="84">
+      <formula>AND($A4&lt;&gt;"",$L5&gt;$M5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M4:N4">
+    <cfRule type="expression" dxfId="29" priority="88">
+      <formula>AND(#REF!&lt;&gt;"",$M4&gt;$N4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M4:N6">
+    <cfRule type="expression" dxfId="28" priority="33">
+      <formula>$M4&gt;$N4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:N200">
+    <cfRule type="expression" dxfId="27" priority="87">
+      <formula>AND($A4&lt;&gt;"",$M5&gt;$N5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N4:O4">
+    <cfRule type="expression" dxfId="26" priority="90">
+      <formula>AND(#REF!&lt;&gt;"",$N4&gt;$O4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N5:O200">
+    <cfRule type="expression" dxfId="25" priority="89">
+      <formula>AND($A4&lt;&gt;"",$N5&gt;$O5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O4:P4">
+    <cfRule type="expression" dxfId="24" priority="92">
+      <formula>AND(#REF!&lt;&gt;"",$O4&gt;$P4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:P200">
+    <cfRule type="expression" dxfId="23" priority="273">
+      <formula>AND($A4&lt;&gt;"",$O5&gt;$P5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q4:R4">
+    <cfRule type="expression" dxfId="22" priority="94">
+      <formula>AND(#REF!&lt;&gt;"",$Q4&gt;$R4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q5:R200">
+    <cfRule type="expression" dxfId="21" priority="274">
+      <formula>AND($A4&lt;&gt;"",$Q5&gt;$R5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="expression" dxfId="20" priority="15">
+      <formula>$G9&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="expression" dxfId="19" priority="20">
+      <formula>AND($A9&lt;&gt;"",#REF!&gt;$G9)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="21">
+      <formula>AND($A9&lt;&gt;"",$G9&gt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9">
+    <cfRule type="expression" dxfId="17" priority="16">
+      <formula>$H9&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9">
+    <cfRule type="expression" dxfId="16" priority="18">
+      <formula>AND($A9&lt;&gt;"",#REF!&gt;$H9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I9">
+    <cfRule type="expression" dxfId="15" priority="17">
+      <formula>$I9&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I9">
+    <cfRule type="expression" dxfId="14" priority="19">
+      <formula>AND($A9&lt;&gt;"",#REF!&gt;$I9)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="47" priority="214">
+    <cfRule type="expression" dxfId="13" priority="8">
+      <formula>$G3&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3">
+    <cfRule type="expression" dxfId="12" priority="13">
       <formula>AND($A3&lt;&gt;"",#REF!&gt;$G3)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="46" priority="215">
+    <cfRule type="expression" dxfId="11" priority="14">
       <formula>AND($A3&lt;&gt;"",$G3&gt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4:G199">
-    <cfRule type="expression" dxfId="45" priority="216">
-      <formula>AND($A4&lt;&gt;"",OR($F4="",#REF!=""))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="44" priority="217">
-      <formula>#REF!&gt;$G4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:H199">
-    <cfRule type="expression" dxfId="43" priority="23">
-      <formula>AND($A4&lt;&gt;"",$G4&gt;$H4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:I8 A9:I199 G3:L3 A3:D8">
-    <cfRule type="expression" dxfId="42" priority="13">
-      <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:L3 A3:D8 G4:I8 A9:I199">
-    <cfRule type="expression" dxfId="41" priority="14">
-      <formula>AND($A3&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H3">
-    <cfRule type="expression" dxfId="40" priority="35">
-      <formula>$H2&gt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3 H4:I199">
-    <cfRule type="expression" dxfId="39" priority="227">
-      <formula>AND($A3&lt;&gt;"",$H3&gt;$I3)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H3">
-    <cfRule type="expression" dxfId="38" priority="140">
+    <cfRule type="expression" dxfId="10" priority="9">
+      <formula>$H3&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" dxfId="9" priority="11">
       <formula>AND($A3&lt;&gt;"",#REF!&gt;$H3)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4:I199">
-    <cfRule type="expression" dxfId="37" priority="9">
-      <formula>$H4&gt;$I4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I3">
-    <cfRule type="expression" dxfId="36" priority="37">
-      <formula>$I2&gt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="35" priority="183">
+    <cfRule type="expression" dxfId="8" priority="10">
+      <formula>$I3&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3">
+    <cfRule type="expression" dxfId="7" priority="12">
       <formula>AND($A3&lt;&gt;"",#REF!&gt;$I3)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I199">
-    <cfRule type="expression" dxfId="34" priority="231">
-      <formula>AND($A3&lt;&gt;"",$I3&gt;#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3:J200">
-    <cfRule type="expression" dxfId="33" priority="232">
-      <formula>AND($A3&lt;&gt;"",#REF!&gt;$J3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J200">
-    <cfRule type="expression" dxfId="32" priority="88">
-      <formula>#REF!&gt;$J5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4:K4">
-    <cfRule type="expression" dxfId="31" priority="61">
-      <formula>AND(#REF!&lt;&gt;"",$J4&gt;$K4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:K7 J8:J10 J11:K200">
-    <cfRule type="expression" dxfId="30" priority="102">
-      <formula>AND($A4&lt;&gt;"",$J5&gt;$K5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4:O4">
-    <cfRule type="expression" dxfId="29" priority="52">
-      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="53">
-      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:O7 J8:J10 L8:O10 J11:O200">
-    <cfRule type="expression" dxfId="27" priority="51">
-      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:O7 L8:O10 J11:O200 J8:J10">
-    <cfRule type="expression" dxfId="26" priority="50">
-      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4:R4">
-    <cfRule type="expression" dxfId="25" priority="56">
-      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="57">
-      <formula>AND(#REF!&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:R7 J8:J10 L8:R10 J11:R200">
-    <cfRule type="expression" dxfId="23" priority="55">
-      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="54">
-      <formula>AND($A4&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K9:K10">
-    <cfRule type="expression" dxfId="21" priority="236">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="20" priority="237">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="238">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="239">
-      <formula>AND($A7&lt;&gt;"",MOD(ROW(),2)=0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="17" priority="240">
-      <formula>$K9&gt;$L8</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="241">
-      <formula>AND($A7&lt;&gt;"",$J8&gt;$K9)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="242">
-      <formula>AND($A7&lt;&gt;"",$K9&gt;$L8)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3:L3">
-    <cfRule type="expression" dxfId="14" priority="243">
-      <formula>AND($A3&lt;&gt;"",$K3&gt;$L3)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K4:L4">
-    <cfRule type="expression" dxfId="13" priority="64">
-      <formula>AND(#REF!&lt;&gt;"",$K4&gt;$L4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K4:L7 L8:L10 K11:L200">
-    <cfRule type="expression" dxfId="12" priority="11">
-      <formula>$K4&gt;$L4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K5:L7 L8:L10 K11:L200">
-    <cfRule type="expression" dxfId="11" priority="62">
-      <formula>AND($A4&lt;&gt;"",$K5&gt;$L5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:M4">
-    <cfRule type="expression" dxfId="10" priority="65">
-      <formula>AND(#REF!&lt;&gt;"",$L4&gt;$M4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L5:M200">
-    <cfRule type="expression" dxfId="9" priority="63">
-      <formula>AND($A4&lt;&gt;"",$L5&gt;$M5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M4:N4">
-    <cfRule type="expression" dxfId="8" priority="67">
-      <formula>AND(#REF!&lt;&gt;"",$M4&gt;$N4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M4:N6">
-    <cfRule type="expression" dxfId="7" priority="12">
-      <formula>$M4&gt;$N4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M5:N200">
-    <cfRule type="expression" dxfId="6" priority="66">
-      <formula>AND($A4&lt;&gt;"",$M5&gt;$N5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N4:O4">
-    <cfRule type="expression" dxfId="5" priority="69">
-      <formula>AND(#REF!&lt;&gt;"",$N4&gt;$O4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N5:O200">
-    <cfRule type="expression" dxfId="4" priority="68">
-      <formula>AND($A4&lt;&gt;"",$N5&gt;$O5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O4:P4">
-    <cfRule type="expression" dxfId="3" priority="71">
-      <formula>AND(#REF!&lt;&gt;"",$O4&gt;$P4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O5:P200">
-    <cfRule type="expression" dxfId="2" priority="252">
-      <formula>AND($A4&lt;&gt;"",$O5&gt;$P5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q4:R4">
-    <cfRule type="expression" dxfId="1" priority="73">
-      <formula>AND(#REF!&lt;&gt;"",$Q4&gt;$R4)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q5:R200">
-    <cfRule type="expression" dxfId="0" priority="253">
-      <formula>AND($A4&lt;&gt;"",$Q5&gt;$R5)</formula>
+  <conditionalFormatting sqref="G4">
+    <cfRule type="expression" dxfId="6" priority="1">
+      <formula>$G4&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4">
+    <cfRule type="expression" dxfId="5" priority="6">
+      <formula>AND($A4&lt;&gt;"",#REF!&gt;$G4)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="7">
+      <formula>AND($A4&lt;&gt;"",$G4&gt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>$H4&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="expression" dxfId="2" priority="4">
+      <formula>AND($A4&lt;&gt;"",#REF!&gt;$H4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4">
+    <cfRule type="expression" dxfId="1" priority="3">
+      <formula>$I4&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4">
+    <cfRule type="expression" dxfId="0" priority="5">
+      <formula>AND($A4&lt;&gt;"",#REF!&gt;$I4)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" sqref="K9:K10 L8:R10 J8:J10 J11:R200 J4:R7 G3:L3 E2:F2 G2:I200 E9:E199 F9:F200 C3:C8 D7:D199" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" sqref="K9:K10 L8:R10 J8:J10 J11:R200 J4:R7 E15:E199 F15:F200 D13:D199 J3:L3 C3:C14 E2:I2 G3:I200 D8:D9" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="E3:E8" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="E3:E14" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"King,Queen,Rook,Bishop,Knight,Pawn"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>